<commit_message>
Ajustar busqueda de paginas prehechas
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://accmotos-my.sharepoint.com/personal/analista_ecommerce_accemotos_com/Documents/Catalogo Skill/Generar_paginas/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://accmotos-my.sharepoint.com/personal/analista_ecommerce_accemotos_com/Documents/Catalogo Skill/accemotos-catalogo-pdf-railway/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="34" documentId="13_ncr:1_{10669B08-BB66-4135-A5E3-9E2DACEF6155}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{008D2313-4DC3-4905-A9D0-272404FE8575}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="13_ncr:1_{10669B08-BB66-4135-A5E3-9E2DACEF6155}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{78D2CC38-B7ED-42B1-88F7-FB29AFE456CF}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4372" uniqueCount="687">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4373" uniqueCount="687">
   <si>
     <t>INVENTARIO</t>
   </si>
@@ -2446,6 +2446,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED19A6D8-9765-4D8B-A3EA-1BB5203692F5}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:L546"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
@@ -2490,7 +2491,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>16867</v>
       </c>
@@ -2528,7 +2529,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>19110</v>
       </c>
@@ -2566,7 +2567,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>15441</v>
       </c>
@@ -2604,7 +2605,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>9901</v>
       </c>
@@ -2642,7 +2643,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>12662</v>
       </c>
@@ -2680,7 +2681,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>16844</v>
       </c>
@@ -2718,7 +2719,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>17222</v>
       </c>
@@ -2756,7 +2757,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>17223</v>
       </c>
@@ -2794,7 +2795,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>17225</v>
       </c>
@@ -2832,7 +2833,7 @@
         <v>684</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>17224</v>
       </c>
@@ -2870,7 +2871,7 @@
         <v>684</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>17220</v>
       </c>
@@ -2908,7 +2909,7 @@
         <v>685</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>17221</v>
       </c>
@@ -2946,7 +2947,7 @@
         <v>685</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>17371</v>
       </c>
@@ -2984,7 +2985,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>17366</v>
       </c>
@@ -3022,7 +3023,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="16" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>17365</v>
       </c>
@@ -3060,7 +3061,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="17" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>17367</v>
       </c>
@@ -3098,7 +3099,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="18" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>17364</v>
       </c>
@@ -3136,7 +3137,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="19" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>17407</v>
       </c>
@@ -3174,7 +3175,7 @@
         <v>504</v>
       </c>
     </row>
-    <row r="20" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>17386</v>
       </c>
@@ -3212,7 +3213,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="21" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>17404</v>
       </c>
@@ -3250,7 +3251,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="22" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>17485</v>
       </c>
@@ -3288,7 +3289,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="23" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>17486</v>
       </c>
@@ -3326,7 +3327,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="24" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>17483</v>
       </c>
@@ -3364,7 +3365,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="25" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>17481</v>
       </c>
@@ -3402,7 +3403,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="26" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>17482</v>
       </c>
@@ -3440,7 +3441,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="27" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>17488</v>
       </c>
@@ -3478,7 +3479,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="28" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>17489</v>
       </c>
@@ -3516,7 +3517,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="29" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>12861</v>
       </c>
@@ -3554,7 +3555,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="30" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>9362</v>
       </c>
@@ -3592,7 +3593,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="31" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>17043</v>
       </c>
@@ -3630,7 +3631,7 @@
         <v>512</v>
       </c>
     </row>
-    <row r="32" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>17044</v>
       </c>
@@ -3668,7 +3669,7 @@
         <v>512</v>
       </c>
     </row>
-    <row r="33" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>17041</v>
       </c>
@@ -3706,7 +3707,7 @@
         <v>512</v>
       </c>
     </row>
-    <row r="34" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>17042</v>
       </c>
@@ -3744,7 +3745,7 @@
         <v>512</v>
       </c>
     </row>
-    <row r="35" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>17039</v>
       </c>
@@ -3782,7 +3783,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="36" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>17038</v>
       </c>
@@ -3820,7 +3821,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="37" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>17037</v>
       </c>
@@ -3858,7 +3859,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="38" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>17040</v>
       </c>
@@ -3896,7 +3897,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="39" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>17033</v>
       </c>
@@ -3934,7 +3935,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="40" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>17034</v>
       </c>
@@ -3972,7 +3973,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="41" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>17035</v>
       </c>
@@ -4010,7 +4011,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="42" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>17036</v>
       </c>
@@ -4048,7 +4049,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="43" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>674</v>
       </c>
@@ -4086,7 +4087,7 @@
         <v>515</v>
       </c>
     </row>
-    <row r="44" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>17251</v>
       </c>
@@ -4124,7 +4125,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="45" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>9264</v>
       </c>
@@ -4162,7 +4163,7 @@
         <v>517</v>
       </c>
     </row>
-    <row r="46" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>16628</v>
       </c>
@@ -4200,7 +4201,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="47" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>17240</v>
       </c>
@@ -4238,7 +4239,7 @@
         <v>519</v>
       </c>
     </row>
-    <row r="48" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>17244</v>
       </c>
@@ -4276,7 +4277,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="49" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>17237</v>
       </c>
@@ -4314,7 +4315,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="50" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>17236</v>
       </c>
@@ -4352,7 +4353,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="51" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>10436</v>
       </c>
@@ -4390,7 +4391,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="52" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>10437</v>
       </c>
@@ -4428,7 +4429,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="53" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>17925</v>
       </c>
@@ -4466,7 +4467,7 @@
         <v>523</v>
       </c>
     </row>
-    <row r="54" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54">
         <v>17926</v>
       </c>
@@ -4504,7 +4505,7 @@
         <v>523</v>
       </c>
     </row>
-    <row r="55" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55">
         <v>17053</v>
       </c>
@@ -4542,7 +4543,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="56" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A56">
         <v>17923</v>
       </c>
@@ -4580,7 +4581,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="57" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A57">
         <v>17843</v>
       </c>
@@ -4618,7 +4619,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="58" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A58">
         <v>17844</v>
       </c>
@@ -4656,7 +4657,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="59" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A59">
         <v>17905</v>
       </c>
@@ -4694,7 +4695,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="60" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A60">
         <v>17908</v>
       </c>
@@ -4732,7 +4733,7 @@
         <v>527</v>
       </c>
     </row>
-    <row r="61" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A61">
         <v>17914</v>
       </c>
@@ -4770,7 +4771,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="62" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A62">
         <v>17911</v>
       </c>
@@ -4808,7 +4809,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="63" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A63">
         <v>16853</v>
       </c>
@@ -4846,7 +4847,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="64" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A64">
         <v>16053</v>
       </c>
@@ -4884,7 +4885,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="65" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A65">
         <v>16849</v>
       </c>
@@ -4922,7 +4923,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="66" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A66">
         <v>17344</v>
       </c>
@@ -4960,7 +4961,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="67" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A67">
         <v>17343</v>
       </c>
@@ -4998,7 +4999,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="68" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A68">
         <v>17346</v>
       </c>
@@ -5036,7 +5037,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="69" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A69">
         <v>17345</v>
       </c>
@@ -5074,7 +5075,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="70" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A70">
         <v>17347</v>
       </c>
@@ -5112,7 +5113,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="71" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A71">
         <v>17349</v>
       </c>
@@ -5150,7 +5151,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="72" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A72">
         <v>17348</v>
       </c>
@@ -5188,7 +5189,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="73" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A73">
         <v>16647</v>
       </c>
@@ -5226,7 +5227,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="74" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74">
         <v>16652</v>
       </c>
@@ -5264,7 +5265,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="75" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75">
         <v>16651</v>
       </c>
@@ -5302,7 +5303,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="76" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A76">
         <v>17800</v>
       </c>
@@ -5340,7 +5341,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="77" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A77">
         <v>17801</v>
       </c>
@@ -5378,7 +5379,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="78" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A78">
         <v>17802</v>
       </c>
@@ -5416,7 +5417,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="79" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A79">
         <v>17798</v>
       </c>
@@ -5454,7 +5455,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="80" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80">
         <v>17781</v>
       </c>
@@ -5492,7 +5493,7 @@
         <v>538</v>
       </c>
     </row>
-    <row r="81" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A81">
         <v>17786</v>
       </c>
@@ -5530,7 +5531,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="82" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A82">
         <v>17787</v>
       </c>
@@ -5568,7 +5569,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="83" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A83">
         <v>17788</v>
       </c>
@@ -5606,7 +5607,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="84" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A84">
         <v>17784</v>
       </c>
@@ -5644,7 +5645,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="85" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A85">
         <v>17785</v>
       </c>
@@ -5682,7 +5683,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="86" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A86">
         <v>17775</v>
       </c>
@@ -5720,7 +5721,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="87" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A87">
         <v>17776</v>
       </c>
@@ -5758,7 +5759,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="88" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A88">
         <v>17777</v>
       </c>
@@ -5796,7 +5797,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="89" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A89">
         <v>17778</v>
       </c>
@@ -5834,7 +5835,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="90" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A90">
         <v>17779</v>
       </c>
@@ -5872,7 +5873,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="91" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A91">
         <v>19001</v>
       </c>
@@ -5910,7 +5911,7 @@
         <v>543</v>
       </c>
     </row>
-    <row r="92" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A92">
         <v>19002</v>
       </c>
@@ -5948,7 +5949,7 @@
         <v>543</v>
       </c>
     </row>
-    <row r="93" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A93">
         <v>19003</v>
       </c>
@@ -5986,7 +5987,7 @@
         <v>543</v>
       </c>
     </row>
-    <row r="94" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A94">
         <v>17070</v>
       </c>
@@ -6024,7 +6025,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="95" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A95">
         <v>17071</v>
       </c>
@@ -6062,7 +6063,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="96" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A96">
         <v>17080</v>
       </c>
@@ -6100,7 +6101,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="97" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A97">
         <v>17084</v>
       </c>
@@ -6138,7 +6139,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="98" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A98">
         <v>17013</v>
       </c>
@@ -6176,7 +6177,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="99" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A99">
         <v>17066</v>
       </c>
@@ -6214,7 +6215,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="100" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A100">
         <v>17076</v>
       </c>
@@ -6252,7 +6253,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="101" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A101">
         <v>17073</v>
       </c>
@@ -6290,7 +6291,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="102" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A102">
         <v>17086</v>
       </c>
@@ -6328,7 +6329,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="103" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A103">
         <v>17093</v>
       </c>
@@ -6366,7 +6367,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="104" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A104">
         <v>17092</v>
       </c>
@@ -6404,7 +6405,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="105" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A105">
         <v>16658</v>
       </c>
@@ -6442,7 +6443,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="106" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A106">
         <v>16657</v>
       </c>
@@ -6480,7 +6481,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="107" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A107">
         <v>16654</v>
       </c>
@@ -6556,7 +6557,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="109" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A109">
         <v>6807</v>
       </c>
@@ -6594,7 +6595,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="110" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A110">
         <v>6808</v>
       </c>
@@ -6632,7 +6633,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="111" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A111">
         <v>17341</v>
       </c>
@@ -6670,7 +6671,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="112" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A112">
         <v>17339</v>
       </c>
@@ -6708,7 +6709,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="113" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A113">
         <v>17338</v>
       </c>
@@ -6746,7 +6747,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="114" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A114">
         <v>17337</v>
       </c>
@@ -6784,7 +6785,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="115" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A115">
         <v>17340</v>
       </c>
@@ -6822,7 +6823,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="116" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A116">
         <v>6810</v>
       </c>
@@ -6860,7 +6861,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="117" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A117">
         <v>6809</v>
       </c>
@@ -6898,7 +6899,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="118" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A118">
         <v>6811</v>
       </c>
@@ -6936,7 +6937,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="119" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A119">
         <v>15512</v>
       </c>
@@ -6974,7 +6975,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="120" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A120">
         <v>16273</v>
       </c>
@@ -7012,7 +7013,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="121" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A121">
         <v>16275</v>
       </c>
@@ -7050,7 +7051,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="122" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A122">
         <v>16276</v>
       </c>
@@ -7088,7 +7089,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="123" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A123">
         <v>17335</v>
       </c>
@@ -7126,7 +7127,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="124" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A124">
         <v>17334</v>
       </c>
@@ -7164,7 +7165,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="125" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A125">
         <v>17327</v>
       </c>
@@ -7202,7 +7203,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="126" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A126">
         <v>17325</v>
       </c>
@@ -7240,7 +7241,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="127" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A127">
         <v>17326</v>
       </c>
@@ -7278,7 +7279,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="128" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A128">
         <v>17330</v>
       </c>
@@ -7316,7 +7317,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="129" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A129">
         <v>17328</v>
       </c>
@@ -7354,7 +7355,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="130" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A130">
         <v>17329</v>
       </c>
@@ -7392,7 +7393,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="131" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A131">
         <v>17333</v>
       </c>
@@ -7430,7 +7431,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="132" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A132">
         <v>17332</v>
       </c>
@@ -7468,7 +7469,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="133" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A133">
         <v>17331</v>
       </c>
@@ -7506,7 +7507,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="134" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A134">
         <v>17323</v>
       </c>
@@ -7544,7 +7545,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="135" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A135">
         <v>17321</v>
       </c>
@@ -7582,7 +7583,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="136" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A136">
         <v>17322</v>
       </c>
@@ -7620,7 +7621,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="137" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A137">
         <v>17320</v>
       </c>
@@ -7658,7 +7659,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="138" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A138">
         <v>17318</v>
       </c>
@@ -7696,7 +7697,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="139" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A139">
         <v>17317</v>
       </c>
@@ -7734,7 +7735,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="140" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A140">
         <v>17319</v>
       </c>
@@ -7772,7 +7773,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="141" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A141">
         <v>14687</v>
       </c>
@@ -7810,7 +7811,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="142" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A142">
         <v>14685</v>
       </c>
@@ -7848,7 +7849,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="143" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A143">
         <v>14690</v>
       </c>
@@ -7886,7 +7887,7 @@
         <v>686</v>
       </c>
     </row>
-    <row r="144" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A144">
         <v>17493</v>
       </c>
@@ -7924,7 +7925,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="145" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A145">
         <v>17491</v>
       </c>
@@ -7962,7 +7963,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="146" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A146">
         <v>17492</v>
       </c>
@@ -8000,7 +8001,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="147" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A147">
         <v>12658</v>
       </c>
@@ -8038,7 +8039,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="148" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A148">
         <v>15319</v>
       </c>
@@ -8076,7 +8077,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="149" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A149">
         <v>15321</v>
       </c>
@@ -8114,7 +8115,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="150" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A150">
         <v>17497</v>
       </c>
@@ -8152,7 +8153,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="151" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A151">
         <v>17495</v>
       </c>
@@ -8190,7 +8191,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="152" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A152">
         <v>17494</v>
       </c>
@@ -8228,7 +8229,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="153" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A153">
         <v>17496</v>
       </c>
@@ -8266,7 +8267,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="154" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A154">
         <v>17503</v>
       </c>
@@ -8304,7 +8305,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="155" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A155">
         <v>17502</v>
       </c>
@@ -8342,7 +8343,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="156" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A156">
         <v>17504</v>
       </c>
@@ -8380,7 +8381,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="157" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A157">
         <v>17500</v>
       </c>
@@ -8418,7 +8419,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="158" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A158">
         <v>17498</v>
       </c>
@@ -8456,7 +8457,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="159" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A159">
         <v>17532</v>
       </c>
@@ -8494,7 +8495,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="160" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A160">
         <v>17499</v>
       </c>
@@ -8532,7 +8533,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="161" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A161">
         <v>16280</v>
       </c>
@@ -8570,7 +8571,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="162" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A162">
         <v>16285</v>
       </c>
@@ -8608,7 +8609,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="163" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A163">
         <v>16282</v>
       </c>
@@ -8646,7 +8647,7 @@
         <v>574</v>
       </c>
     </row>
-    <row r="164" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A164">
         <v>16249</v>
       </c>
@@ -8684,7 +8685,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="165" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A165">
         <v>17312</v>
       </c>
@@ -8722,7 +8723,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="166" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A166">
         <v>17310</v>
       </c>
@@ -8760,7 +8761,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="167" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A167">
         <v>17309</v>
       </c>
@@ -8798,7 +8799,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="168" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A168">
         <v>17315</v>
       </c>
@@ -8836,7 +8837,7 @@
         <v>577</v>
       </c>
     </row>
-    <row r="169" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A169">
         <v>17314</v>
       </c>
@@ -8874,7 +8875,7 @@
         <v>577</v>
       </c>
     </row>
-    <row r="170" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A170">
         <v>17313</v>
       </c>
@@ -8912,7 +8913,7 @@
         <v>577</v>
       </c>
     </row>
-    <row r="171" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A171">
         <v>16261</v>
       </c>
@@ -8950,7 +8951,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="172" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A172">
         <v>16259</v>
       </c>
@@ -8988,7 +8989,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="173" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A173">
         <v>16260</v>
       </c>
@@ -9026,7 +9027,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="174" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A174">
         <v>16256</v>
       </c>
@@ -9064,7 +9065,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="175" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A175">
         <v>11418</v>
       </c>
@@ -9710,7 +9711,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="192" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A192">
         <v>16296</v>
       </c>
@@ -9748,7 +9749,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="193" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A193">
         <v>16294</v>
       </c>
@@ -9786,7 +9787,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="194" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A194">
         <v>16293</v>
       </c>
@@ -9824,7 +9825,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="195" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A195">
         <v>16292</v>
       </c>
@@ -9862,7 +9863,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="196" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A196">
         <v>16295</v>
       </c>
@@ -9900,7 +9901,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="197" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A197">
         <v>13102</v>
       </c>
@@ -9938,7 +9939,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="198" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A198">
         <v>13100</v>
       </c>
@@ -9976,7 +9977,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="199" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A199">
         <v>13099</v>
       </c>
@@ -10014,7 +10015,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="200" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A200">
         <v>16298</v>
       </c>
@@ -10052,7 +10053,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="201" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A201">
         <v>13101</v>
       </c>
@@ -10090,7 +10091,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="202" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A202">
         <v>16297</v>
       </c>
@@ -10128,7 +10129,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="203" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A203">
         <v>16304</v>
       </c>
@@ -10166,7 +10167,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="204" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A204">
         <v>16302</v>
       </c>
@@ -10204,7 +10205,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="205" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A205">
         <v>16301</v>
       </c>
@@ -10242,7 +10243,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="206" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A206">
         <v>16300</v>
       </c>
@@ -10280,7 +10281,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="207" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A207">
         <v>16303</v>
       </c>
@@ -10318,7 +10319,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="208" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A208">
         <v>16299</v>
       </c>
@@ -10356,7 +10357,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="209" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A209">
         <v>16310</v>
       </c>
@@ -10394,7 +10395,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="210" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A210">
         <v>16308</v>
       </c>
@@ -10432,7 +10433,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="211" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A211">
         <v>16307</v>
       </c>
@@ -10470,7 +10471,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="212" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A212">
         <v>16306</v>
       </c>
@@ -10508,7 +10509,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="213" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A213">
         <v>16309</v>
       </c>
@@ -10546,7 +10547,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="214" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A214">
         <v>16305</v>
       </c>
@@ -10584,7 +10585,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="215" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A215">
         <v>13119</v>
       </c>
@@ -10622,7 +10623,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="216" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A216">
         <v>13117</v>
       </c>
@@ -10660,7 +10661,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="217" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A217">
         <v>13116</v>
       </c>
@@ -10698,7 +10699,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="218" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A218">
         <v>13115</v>
       </c>
@@ -10736,7 +10737,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="219" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A219">
         <v>13118</v>
       </c>
@@ -10774,7 +10775,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="220" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A220">
         <v>16290</v>
       </c>
@@ -10812,7 +10813,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="221" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A221">
         <v>14235</v>
       </c>
@@ -10850,7 +10851,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="222" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A222">
         <v>14232</v>
       </c>
@@ -10888,7 +10889,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="223" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A223">
         <v>14233</v>
       </c>
@@ -10926,7 +10927,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="224" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A224">
         <v>14231</v>
       </c>
@@ -10964,7 +10965,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="225" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A225">
         <v>14234</v>
       </c>
@@ -11002,7 +11003,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="226" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A226">
         <v>14735</v>
       </c>
@@ -11040,7 +11041,7 @@
         <v>596</v>
       </c>
     </row>
-    <row r="227" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A227">
         <v>14698</v>
       </c>
@@ -11078,7 +11079,7 @@
         <v>596</v>
       </c>
     </row>
-    <row r="228" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A228">
         <v>14278</v>
       </c>
@@ -11116,7 +11117,7 @@
         <v>669</v>
       </c>
     </row>
-    <row r="229" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A229">
         <v>14280</v>
       </c>
@@ -11154,7 +11155,7 @@
         <v>669</v>
       </c>
     </row>
-    <row r="230" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A230">
         <v>14279</v>
       </c>
@@ -11192,7 +11193,7 @@
         <v>669</v>
       </c>
     </row>
-    <row r="231" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A231">
         <v>14722</v>
       </c>
@@ -11230,7 +11231,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="232" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A232">
         <v>14274</v>
       </c>
@@ -11268,7 +11269,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="233" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A233">
         <v>14275</v>
       </c>
@@ -11306,7 +11307,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="234" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A234">
         <v>14255</v>
       </c>
@@ -11344,7 +11345,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="235" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A235">
         <v>14254</v>
       </c>
@@ -11382,7 +11383,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="236" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A236">
         <v>14253</v>
       </c>
@@ -11420,7 +11421,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="237" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A237">
         <v>14252</v>
       </c>
@@ -11458,7 +11459,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="238" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A238">
         <v>14251</v>
       </c>
@@ -11496,7 +11497,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="239" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A239">
         <v>14250</v>
       </c>
@@ -11534,7 +11535,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="240" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A240">
         <v>14244</v>
       </c>
@@ -11572,7 +11573,7 @@
         <v>670</v>
       </c>
     </row>
-    <row r="241" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A241">
         <v>14245</v>
       </c>
@@ -11610,7 +11611,7 @@
         <v>601</v>
       </c>
     </row>
-    <row r="242" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A242">
         <v>14248</v>
       </c>
@@ -11648,7 +11649,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="243" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A243">
         <v>14247</v>
       </c>
@@ -11686,7 +11687,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="244" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A244">
         <v>14249</v>
       </c>
@@ -11724,7 +11725,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="245" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A245">
         <v>14268</v>
       </c>
@@ -11762,7 +11763,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="246" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A246">
         <v>14267</v>
       </c>
@@ -11800,7 +11801,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="247" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A247">
         <v>14265</v>
       </c>
@@ -11838,7 +11839,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="248" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A248">
         <v>15430</v>
       </c>
@@ -11876,7 +11877,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="249" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A249">
         <v>15428</v>
       </c>
@@ -11914,7 +11915,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="250" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A250">
         <v>15427</v>
       </c>
@@ -11952,7 +11953,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="251" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A251">
         <v>17274</v>
       </c>
@@ -11990,7 +11991,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="252" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A252">
         <v>14323</v>
       </c>
@@ -12028,7 +12029,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="253" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A253">
         <v>14312</v>
       </c>
@@ -12066,7 +12067,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="254" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A254">
         <v>16333</v>
       </c>
@@ -12902,7 +12903,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="276" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A276">
         <v>17295</v>
       </c>
@@ -12940,7 +12941,7 @@
         <v>619</v>
       </c>
     </row>
-    <row r="277" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A277">
         <v>17296</v>
       </c>
@@ -12978,7 +12979,7 @@
         <v>619</v>
       </c>
     </row>
-    <row r="278" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A278">
         <v>17297</v>
       </c>
@@ -13016,7 +13017,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="279" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A279">
         <v>17298</v>
       </c>
@@ -13054,7 +13055,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="280" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A280">
         <v>17288</v>
       </c>
@@ -13092,7 +13093,7 @@
         <v>621</v>
       </c>
     </row>
-    <row r="281" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A281">
         <v>17302</v>
       </c>
@@ -13130,7 +13131,7 @@
         <v>679</v>
       </c>
     </row>
-    <row r="282" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A282">
         <v>16951</v>
       </c>
@@ -13168,7 +13169,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="283" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A283">
         <v>16952</v>
       </c>
@@ -13206,7 +13207,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="284" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A284">
         <v>17299</v>
       </c>
@@ -13244,7 +13245,7 @@
         <v>623</v>
       </c>
     </row>
-    <row r="285" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A285">
         <v>17300</v>
       </c>
@@ -13282,7 +13283,7 @@
         <v>623</v>
       </c>
     </row>
-    <row r="286" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A286">
         <v>17293</v>
       </c>
@@ -13320,7 +13321,7 @@
         <v>624</v>
       </c>
     </row>
-    <row r="287" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A287">
         <v>17434</v>
       </c>
@@ -13358,7 +13359,7 @@
         <v>625</v>
       </c>
     </row>
-    <row r="288" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A288">
         <v>17435</v>
       </c>
@@ -13396,7 +13397,7 @@
         <v>625</v>
       </c>
     </row>
-    <row r="289" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A289">
         <v>17436</v>
       </c>
@@ -13434,7 +13435,7 @@
         <v>625</v>
       </c>
     </row>
-    <row r="290" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A290">
         <v>17417</v>
       </c>
@@ -13472,7 +13473,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="291" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A291">
         <v>17418</v>
       </c>
@@ -13510,7 +13511,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="292" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A292">
         <v>17419</v>
       </c>
@@ -13548,7 +13549,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="293" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A293">
         <v>17427</v>
       </c>
@@ -13586,7 +13587,7 @@
         <v>627</v>
       </c>
     </row>
-    <row r="294" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A294">
         <v>17428</v>
       </c>
@@ -13624,7 +13625,7 @@
         <v>627</v>
       </c>
     </row>
-    <row r="295" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A295">
         <v>17411</v>
       </c>
@@ -13662,7 +13663,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="296" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A296">
         <v>17412</v>
       </c>
@@ -13700,7 +13701,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="297" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A297">
         <v>17413</v>
       </c>
@@ -13738,7 +13739,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="298" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A298">
         <v>17429</v>
       </c>
@@ -13776,7 +13777,7 @@
         <v>629</v>
       </c>
     </row>
-    <row r="299" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A299">
         <v>17430</v>
       </c>
@@ -13814,7 +13815,7 @@
         <v>629</v>
       </c>
     </row>
-    <row r="300" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A300">
         <v>17420</v>
       </c>
@@ -13852,7 +13853,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="301" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A301">
         <v>17421</v>
       </c>
@@ -13890,7 +13891,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="302" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A302">
         <v>17422</v>
       </c>
@@ -13928,7 +13929,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="303" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A303">
         <v>17431</v>
       </c>
@@ -13966,7 +13967,7 @@
         <v>631</v>
       </c>
     </row>
-    <row r="304" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A304">
         <v>17432</v>
       </c>
@@ -14004,7 +14005,7 @@
         <v>631</v>
       </c>
     </row>
-    <row r="305" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A305">
         <v>17433</v>
       </c>
@@ -14042,7 +14043,7 @@
         <v>631</v>
       </c>
     </row>
-    <row r="306" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A306">
         <v>17414</v>
       </c>
@@ -14080,7 +14081,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="307" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A307">
         <v>17415</v>
       </c>
@@ -14118,7 +14119,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="308" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A308">
         <v>17416</v>
       </c>
@@ -14156,7 +14157,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="309" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A309">
         <v>17425</v>
       </c>
@@ -14194,7 +14195,7 @@
         <v>633</v>
       </c>
     </row>
-    <row r="310" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A310">
         <v>17426</v>
       </c>
@@ -14232,7 +14233,7 @@
         <v>633</v>
       </c>
     </row>
-    <row r="311" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A311">
         <v>17423</v>
       </c>
@@ -14270,7 +14271,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="312" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A312">
         <v>17424</v>
       </c>
@@ -14308,7 +14309,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="313" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A313">
         <v>17408</v>
       </c>
@@ -14346,7 +14347,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="314" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A314">
         <v>17409</v>
       </c>
@@ -14384,7 +14385,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="315" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A315">
         <v>17410</v>
       </c>
@@ -14422,7 +14423,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="316" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A316">
         <v>17294</v>
       </c>
@@ -14460,7 +14461,7 @@
         <v>636</v>
       </c>
     </row>
-    <row r="317" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A317">
         <v>17289</v>
       </c>
@@ -14498,7 +14499,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="318" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A318">
         <v>17301</v>
       </c>
@@ -14536,7 +14537,7 @@
         <v>638</v>
       </c>
     </row>
-    <row r="319" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A319">
         <v>17278</v>
       </c>
@@ -14574,7 +14575,7 @@
         <v>639</v>
       </c>
     </row>
-    <row r="320" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A320">
         <v>17283</v>
       </c>
@@ -14612,7 +14613,7 @@
         <v>680</v>
       </c>
     </row>
-    <row r="321" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A321">
         <v>16941</v>
       </c>
@@ -14650,7 +14651,7 @@
         <v>640</v>
       </c>
     </row>
-    <row r="322" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A322">
         <v>16942</v>
       </c>
@@ -14688,7 +14689,7 @@
         <v>640</v>
       </c>
     </row>
-    <row r="323" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A323">
         <v>17286</v>
       </c>
@@ -14726,7 +14727,7 @@
         <v>682</v>
       </c>
     </row>
-    <row r="324" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A324">
         <v>17285</v>
       </c>
@@ -14764,7 +14765,7 @@
         <v>682</v>
       </c>
     </row>
-    <row r="325" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A325">
         <v>17287</v>
       </c>
@@ -14802,7 +14803,7 @@
         <v>682</v>
       </c>
     </row>
-    <row r="326" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A326">
         <v>16944</v>
       </c>
@@ -14840,7 +14841,7 @@
         <v>641</v>
       </c>
     </row>
-    <row r="327" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A327">
         <v>16943</v>
       </c>
@@ -14878,7 +14879,7 @@
         <v>641</v>
       </c>
     </row>
-    <row r="328" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A328">
         <v>17840</v>
       </c>
@@ -14916,7 +14917,7 @@
         <v>642</v>
       </c>
     </row>
-    <row r="329" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A329">
         <v>17841</v>
       </c>
@@ -14954,7 +14955,7 @@
         <v>642</v>
       </c>
     </row>
-    <row r="330" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A330">
         <v>17688</v>
       </c>
@@ -14992,7 +14993,7 @@
         <v>643</v>
       </c>
     </row>
-    <row r="331" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A331">
         <v>16939</v>
       </c>
@@ -15030,7 +15031,7 @@
         <v>643</v>
       </c>
     </row>
-    <row r="332" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A332">
         <v>16508</v>
       </c>
@@ -15068,7 +15069,7 @@
         <v>644</v>
       </c>
     </row>
-    <row r="333" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A333">
         <v>16507</v>
       </c>
@@ -15106,7 +15107,7 @@
         <v>644</v>
       </c>
     </row>
-    <row r="334" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A334">
         <v>16509</v>
       </c>
@@ -15144,7 +15145,7 @@
         <v>644</v>
       </c>
     </row>
-    <row r="335" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A335">
         <v>16506</v>
       </c>
@@ -15182,7 +15183,7 @@
         <v>644</v>
       </c>
     </row>
-    <row r="336" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A336">
         <v>9902</v>
       </c>
@@ -15220,7 +15221,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="337" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="337" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A337">
         <v>16677</v>
       </c>
@@ -15258,7 +15259,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="338" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A338">
         <v>14229</v>
       </c>
@@ -15296,7 +15297,7 @@
         <v>645</v>
       </c>
     </row>
-    <row r="339" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A339">
         <v>14730</v>
       </c>
@@ -15334,7 +15335,7 @@
         <v>645</v>
       </c>
     </row>
-    <row r="340" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A340">
         <v>14682</v>
       </c>
@@ -15372,7 +15373,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="341" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A341">
         <v>17270</v>
       </c>
@@ -15410,7 +15411,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="342" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A342">
         <v>17271</v>
       </c>
@@ -15448,7 +15449,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="343" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A343">
         <v>17272</v>
       </c>
@@ -15486,7 +15487,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="344" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="344" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A344">
         <v>14601</v>
       </c>
@@ -17082,7 +17083,7 @@
         <v>653</v>
       </c>
     </row>
-    <row r="386" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="386" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A386">
         <v>15626</v>
       </c>
@@ -17120,7 +17121,7 @@
         <v>654</v>
       </c>
     </row>
-    <row r="387" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="387" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A387">
         <v>15629</v>
       </c>
@@ -17158,7 +17159,7 @@
         <v>655</v>
       </c>
     </row>
-    <row r="388" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="388" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A388">
         <v>17830</v>
       </c>
@@ -17196,7 +17197,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="389" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="389" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A389">
         <v>17831</v>
       </c>
@@ -17234,7 +17235,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="390" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="390" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A390">
         <v>17825</v>
       </c>
@@ -17272,7 +17273,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="391" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="391" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A391">
         <v>17826</v>
       </c>
@@ -17310,7 +17311,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="392" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="392" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A392">
         <v>17827</v>
       </c>
@@ -17348,7 +17349,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="393" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="393" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A393">
         <v>19130</v>
       </c>
@@ -17386,7 +17387,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="394" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="394" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A394">
         <v>19131</v>
       </c>
@@ -17424,7 +17425,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="395" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="395" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A395">
         <v>19132</v>
       </c>
@@ -17462,7 +17463,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="396" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="396" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A396">
         <v>17820</v>
       </c>
@@ -17500,7 +17501,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="397" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="397" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A397">
         <v>17821</v>
       </c>
@@ -17538,7 +17539,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="398" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="398" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A398">
         <v>17828</v>
       </c>
@@ -17576,7 +17577,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="399" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="399" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A399">
         <v>17829</v>
       </c>
@@ -17614,7 +17615,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="400" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="400" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A400">
         <v>17822</v>
       </c>
@@ -17652,7 +17653,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="401" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="401" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A401">
         <v>17823</v>
       </c>
@@ -17690,7 +17691,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="402" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="402" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A402">
         <v>17824</v>
       </c>
@@ -17728,7 +17729,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="403" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="403" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A403">
         <v>17516</v>
       </c>
@@ -17766,7 +17767,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="404" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="404" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A404">
         <v>17514</v>
       </c>
@@ -17804,7 +17805,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="405" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="405" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A405">
         <v>17515</v>
       </c>
@@ -17842,7 +17843,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="406" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="406" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A406">
         <v>17509</v>
       </c>
@@ -17880,7 +17881,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="407" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="407" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A407">
         <v>17510</v>
       </c>
@@ -17918,7 +17919,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="408" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="408" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A408">
         <v>19128</v>
       </c>
@@ -17956,7 +17957,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="409" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="409" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A409">
         <v>19129</v>
       </c>
@@ -17994,7 +17995,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="410" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="410" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A410">
         <v>17525</v>
       </c>
@@ -18032,7 +18033,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="411" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="411" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A411">
         <v>17523</v>
       </c>
@@ -18070,7 +18071,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="412" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="412" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A412">
         <v>17524</v>
       </c>
@@ -18108,7 +18109,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="413" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="413" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A413">
         <v>19124</v>
       </c>
@@ -18146,7 +18147,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="414" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="414" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A414">
         <v>17512</v>
       </c>
@@ -18184,7 +18185,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="415" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="415" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A415">
         <v>17513</v>
       </c>
@@ -18222,7 +18223,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="416" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="416" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A416">
         <v>19126</v>
       </c>
@@ -18260,7 +18261,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="417" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="417" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A417">
         <v>19127</v>
       </c>
@@ -18298,7 +18299,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="418" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="418" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A418">
         <v>17520</v>
       </c>
@@ -18336,7 +18337,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="419" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="419" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A419">
         <v>17521</v>
       </c>
@@ -18374,7 +18375,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="420" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="420" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A420">
         <v>17522</v>
       </c>
@@ -18412,7 +18413,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="421" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="421" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A421">
         <v>17519</v>
       </c>
@@ -18450,7 +18451,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="422" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="422" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A422">
         <v>17517</v>
       </c>
@@ -18488,7 +18489,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="423" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="423" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A423">
         <v>17518</v>
       </c>
@@ -18526,7 +18527,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="424" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="424" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A424">
         <v>17507</v>
       </c>
@@ -18564,7 +18565,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="425" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="425" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A425">
         <v>17508</v>
       </c>
@@ -18602,7 +18603,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="426" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="426" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A426">
         <v>17506</v>
       </c>
@@ -18640,7 +18641,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="427" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="427" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A427">
         <v>17505</v>
       </c>
@@ -18678,7 +18679,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="428" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="428" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A428">
         <v>17527</v>
       </c>
@@ -18716,7 +18717,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="429" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="429" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A429">
         <v>17528</v>
       </c>
@@ -18754,7 +18755,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="430" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="430" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A430">
         <v>17202</v>
       </c>
@@ -18792,7 +18793,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="431" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="431" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A431">
         <v>17203</v>
       </c>
@@ -18830,7 +18831,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="432" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="432" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A432">
         <v>17197</v>
       </c>
@@ -18868,7 +18869,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="433" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="433" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A433">
         <v>17189</v>
       </c>
@@ -18906,7 +18907,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="434" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="434" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A434">
         <v>17188</v>
       </c>
@@ -18944,7 +18945,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="435" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="435" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A435">
         <v>17190</v>
       </c>
@@ -18982,7 +18983,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="436" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="436" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A436">
         <v>17819</v>
       </c>
@@ -19248,7 +19249,7 @@
         <v>658</v>
       </c>
     </row>
-    <row r="443" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="443" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A443">
         <v>16933</v>
       </c>
@@ -19286,7 +19287,7 @@
         <v>659</v>
       </c>
     </row>
-    <row r="444" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="444" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A444">
         <v>16932</v>
       </c>
@@ -19324,7 +19325,7 @@
         <v>659</v>
       </c>
     </row>
-    <row r="445" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="445" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A445">
         <v>16934</v>
       </c>
@@ -19362,7 +19363,7 @@
         <v>659</v>
       </c>
     </row>
-    <row r="446" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="446" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A446">
         <v>16936</v>
       </c>
@@ -19400,7 +19401,7 @@
         <v>660</v>
       </c>
     </row>
-    <row r="447" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="447" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A447">
         <v>16935</v>
       </c>
@@ -19438,7 +19439,7 @@
         <v>660</v>
       </c>
     </row>
-    <row r="448" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="448" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A448">
         <v>16930</v>
       </c>
@@ -19476,7 +19477,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="449" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="449" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A449">
         <v>16929</v>
       </c>
@@ -19514,7 +19515,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="450" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="450" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A450">
         <v>16928</v>
       </c>
@@ -19552,7 +19553,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="451" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="451" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A451">
         <v>13880</v>
       </c>
@@ -19590,7 +19591,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="452" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="452" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A452">
         <v>16842</v>
       </c>
@@ -19628,7 +19629,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="453" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="453" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A453">
         <v>16843</v>
       </c>
@@ -19666,7 +19667,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="454" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="454" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A454">
         <v>19057</v>
       </c>
@@ -19704,7 +19705,7 @@
         <v>661</v>
       </c>
     </row>
-    <row r="455" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="455" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A455">
         <v>19058</v>
       </c>
@@ -19742,7 +19743,7 @@
         <v>661</v>
       </c>
     </row>
-    <row r="456" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="456" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A456">
         <v>19059</v>
       </c>
@@ -19780,7 +19781,7 @@
         <v>662</v>
       </c>
     </row>
-    <row r="457" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="457" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A457">
         <v>19060</v>
       </c>
@@ -19818,7 +19819,7 @@
         <v>662</v>
       </c>
     </row>
-    <row r="458" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="458" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A458">
         <v>16786</v>
       </c>
@@ -19856,7 +19857,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="459" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="459" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A459">
         <v>16788</v>
       </c>
@@ -19894,7 +19895,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="460" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="460" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A460">
         <v>16793</v>
       </c>
@@ -19932,7 +19933,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="461" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="461" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A461">
         <v>16794</v>
       </c>
@@ -19970,7 +19971,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="462" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="462" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A462">
         <v>16796</v>
       </c>
@@ -20008,7 +20009,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="463" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="463" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A463">
         <v>16795</v>
       </c>
@@ -20046,7 +20047,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="464" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="464" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A464">
         <v>19133</v>
       </c>
@@ -20084,7 +20085,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="465" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="465" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A465">
         <v>19134</v>
       </c>
@@ -20122,7 +20123,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="466" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="466" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A466">
         <v>19136</v>
       </c>
@@ -20160,7 +20161,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="467" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="467" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A467">
         <v>19137</v>
       </c>
@@ -20198,7 +20199,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="468" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="468" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A468">
         <v>19139</v>
       </c>
@@ -20236,7 +20237,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="469" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="469" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A469">
         <v>19140</v>
       </c>
@@ -20274,7 +20275,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="470" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="470" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A470">
         <v>19142</v>
       </c>
@@ -20312,7 +20313,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="471" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="471" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A471">
         <v>19144</v>
       </c>
@@ -20350,7 +20351,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="472" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="472" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A472">
         <v>19145</v>
       </c>
@@ -20388,7 +20389,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="473" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="473" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A473">
         <v>19146</v>
       </c>
@@ -20426,7 +20427,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="474" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="474" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A474">
         <v>19148</v>
       </c>
@@ -20464,7 +20465,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="475" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="475" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A475">
         <v>19149</v>
       </c>
@@ -20502,7 +20503,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="476" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="476" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A476">
         <v>19153</v>
       </c>
@@ -20540,7 +20541,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="477" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="477" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A477">
         <v>19154</v>
       </c>
@@ -20578,7 +20579,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="478" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="478" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A478">
         <v>19155</v>
       </c>
@@ -20616,7 +20617,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="479" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="479" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A479">
         <v>19157</v>
       </c>
@@ -20654,7 +20655,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="480" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="480" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A480">
         <v>19158</v>
       </c>
@@ -20692,7 +20693,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="481" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="481" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A481">
         <v>19159</v>
       </c>
@@ -20730,7 +20731,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="482" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="482" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A482">
         <v>19160</v>
       </c>
@@ -20768,7 +20769,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="483" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="483" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A483">
         <v>19161</v>
       </c>
@@ -20806,7 +20807,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="484" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="484" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A484">
         <v>19162</v>
       </c>
@@ -20844,7 +20845,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="485" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="485" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A485">
         <v>19163</v>
       </c>
@@ -20882,7 +20883,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="486" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="486" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A486">
         <v>19164</v>
       </c>
@@ -20920,7 +20921,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="487" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="487" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A487">
         <v>19166</v>
       </c>
@@ -20958,7 +20959,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="488" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="488" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A488">
         <v>19168</v>
       </c>
@@ -20996,7 +20997,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="489" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="489" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A489">
         <v>19170</v>
       </c>
@@ -21034,7 +21035,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="490" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="490" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A490">
         <v>16518</v>
       </c>
@@ -21072,7 +21073,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="491" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="491" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A491">
         <v>16519</v>
       </c>
@@ -21110,7 +21111,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="492" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="492" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A492">
         <v>16520</v>
       </c>
@@ -21126,6 +21127,9 @@
       <c r="E492">
         <v>43</v>
       </c>
+      <c r="F492" t="s">
+        <v>4</v>
+      </c>
       <c r="G492" t="s">
         <v>143</v>
       </c>
@@ -21145,7 +21149,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="493" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="493" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A493">
         <v>17739</v>
       </c>
@@ -21183,7 +21187,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="494" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="494" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A494">
         <v>17740</v>
       </c>
@@ -21221,7 +21225,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="495" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="495" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A495">
         <v>17741</v>
       </c>
@@ -21259,7 +21263,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="496" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="496" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A496">
         <v>17742</v>
       </c>
@@ -21297,7 +21301,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="497" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="497" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A497">
         <v>17743</v>
       </c>
@@ -21335,7 +21339,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="498" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="498" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A498">
         <v>17744</v>
       </c>
@@ -21373,7 +21377,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="499" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="499" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A499">
         <v>17745</v>
       </c>
@@ -21411,7 +21415,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="500" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="500" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A500">
         <v>17746</v>
       </c>
@@ -21449,7 +21453,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="501" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="501" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A501">
         <v>17747</v>
       </c>
@@ -21487,7 +21491,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="502" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="502" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A502">
         <v>17748</v>
       </c>
@@ -21525,7 +21529,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="503" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="503" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A503">
         <v>17749</v>
       </c>
@@ -21563,7 +21567,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="504" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="504" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A504">
         <v>17750</v>
       </c>
@@ -21601,7 +21605,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="505" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="505" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A505">
         <v>17751</v>
       </c>
@@ -21639,7 +21643,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="506" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="506" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A506">
         <v>17752</v>
       </c>
@@ -21677,7 +21681,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="507" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="507" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A507">
         <v>17753</v>
       </c>
@@ -21715,7 +21719,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="508" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="508" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A508">
         <v>17754</v>
       </c>
@@ -21753,7 +21757,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="509" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="509" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A509">
         <v>17755</v>
       </c>
@@ -21791,7 +21795,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="510" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="510" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A510">
         <v>17756</v>
       </c>
@@ -21829,7 +21833,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="511" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="511" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A511">
         <v>17757</v>
       </c>
@@ -21867,7 +21871,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="512" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="512" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A512">
         <v>17758</v>
       </c>
@@ -21905,7 +21909,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="513" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="513" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A513">
         <v>17759</v>
       </c>
@@ -21943,7 +21947,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="514" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="514" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A514">
         <v>17760</v>
       </c>
@@ -21981,7 +21985,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="515" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="515" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A515">
         <v>17761</v>
       </c>
@@ -22019,7 +22023,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="516" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="516" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A516">
         <v>17762</v>
       </c>
@@ -22057,7 +22061,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="517" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="517" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A517">
         <v>17763</v>
       </c>
@@ -22095,7 +22099,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="518" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="518" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A518">
         <v>17764</v>
       </c>
@@ -22133,7 +22137,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="519" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="519" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A519">
         <v>17765</v>
       </c>
@@ -22171,7 +22175,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="520" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="520" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A520">
         <v>17766</v>
       </c>
@@ -22209,7 +22213,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="521" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="521" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A521">
         <v>17767</v>
       </c>
@@ -22247,7 +22251,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="522" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="522" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A522">
         <v>17768</v>
       </c>
@@ -22285,7 +22289,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="523" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="523" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A523">
         <v>17769</v>
       </c>
@@ -22323,7 +22327,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="524" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="524" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A524">
         <v>17770</v>
       </c>
@@ -22361,7 +22365,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="525" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="525" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A525">
         <v>17771</v>
       </c>
@@ -22399,7 +22403,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="526" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="526" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A526">
         <v>17772</v>
       </c>
@@ -22437,7 +22441,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="527" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="527" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A527">
         <v>17773</v>
       </c>
@@ -22475,7 +22479,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="528" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="528" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A528">
         <v>17774</v>
       </c>
@@ -22513,7 +22517,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="529" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="529" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A529">
         <v>16787</v>
       </c>
@@ -22551,7 +22555,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="530" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="530" spans="1:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A530">
         <v>16792</v>
       </c>
@@ -23198,7 +23202,19 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L546" xr:uid="{ED19A6D8-9765-4D8B-A3EA-1BB5203692F5}"/>
+  <autoFilter ref="A1:L546" xr:uid="{ED19A6D8-9765-4D8B-A3EA-1BB5203692F5}">
+    <filterColumn colId="5">
+      <filters>
+        <filter val="XTRONG"/>
+        <filter val="XTRONG GP"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="9">
+      <filters>
+        <filter val="cascos integrales"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <hyperlinks>
     <hyperlink ref="L353" r:id="rId1" display="https://xtronghelmets.com/wp-content/uploads/2026/02/image00026.png,https://xtronghelmets.com/wp-content/uploads/2026/02/image00025.png,https://xtronghelmets.com/wp-content/uploads/2026/02/image00022.png,https://xtronghelmets.com/wp-content/uploads/2025/04/image00072.png" xr:uid="{DF6F3A8E-B34D-4A59-8545-B938A847A8F0}"/>
     <hyperlink ref="L12" r:id="rId2" display="https://xecurohelmets.com/wp-content/uploads/2026/02/XR-003_FLEX-ROJO-NARANJA-BRILLO_VS-AD-GOGLES_xs17220_xm17221_0000_4.png,https://xecurohelmets.com/wp-content/uploads/2026/02/XR-003_FLEX-ROJO-NARANJA-BRILLO_VS-AD-GOGLES_xs17220_xm17221_0001_2.png,https://xecurohelmets.com/wp-content/uploads/2026/02/XR-003_FLEX-ROJO-NARANJA-BRILLO_VS-AD-GOGLES_xs17220_xm17221_0000_3.png,https://xecurohelmets.com/wp-content/uploads/2026/02/XR-003_FLEX-ROJO-NARANJA-BRILLO_VS-AD-GOGLES_xs17220_xm17221_0002_1.png" xr:uid="{EAB28D93-F029-433B-9D75-85EE87CAE4C5}"/>

</xml_diff>